<commit_message>
personnel update & methods edit
</commit_message>
<xml_diff>
--- a/nes-lter-chl-mvco-info.xlsx
+++ b/nes-lter-chl-mvco-info.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28925"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\github\nes-ims\nes-lter-chl-mvco\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kmorkeski\Documents\nes-lter-chl-mvco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C14383-2287-4594-99DC-B020292A4897}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD9A2C12-38AA-4F45-887D-5D89AA211C2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ColumnHeaders" sheetId="1" r:id="rId1"/>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="117">
   <si>
     <t>attributeName</t>
   </si>
@@ -160,9 +160,6 @@
     <t>NSF</t>
   </si>
   <si>
-    <t>OCE-1655686</t>
-  </si>
-  <si>
     <t>creator</t>
   </si>
   <si>
@@ -175,9 +172,6 @@
     <t>contact</t>
   </si>
   <si>
-    <t>metadataProvider</t>
-  </si>
-  <si>
     <t>code</t>
   </si>
   <si>
@@ -193,21 +187,9 @@
     <t>Depth of sample below sea surface http://vocab.nerc.ac.uk/collection/P09/current/DEPH/</t>
   </si>
   <si>
-    <t>Kate</t>
-  </si>
-  <si>
-    <t>Morkeski</t>
-  </si>
-  <si>
-    <t>kmorkeski@whoi.edu</t>
-  </si>
-  <si>
     <t>PI</t>
   </si>
   <si>
-    <t>0000-0002-2903-5851</t>
-  </si>
-  <si>
     <t>Northeast U.S. Continental Shelf</t>
   </si>
   <si>
@@ -377,13 +359,34 @@
   </si>
   <si>
     <t>Taylor</t>
+  </si>
+  <si>
+    <t>OCE-2322676</t>
+  </si>
+  <si>
+    <t>Megan</t>
+  </si>
+  <si>
+    <t>Ferguson</t>
+  </si>
+  <si>
+    <t>megan.ferguson@whoi.edu</t>
+  </si>
+  <si>
+    <t>0009-0002-4496-6600</t>
+  </si>
+  <si>
+    <t>0000-0002-2122-0462</t>
+  </si>
+  <si>
+    <t>0000-0003-0194-7282</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -392,23 +395,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color rgb="FF1D1C1D"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -425,6 +413,12 @@
       <color rgb="FF569CD6"/>
       <name val="Consolas"/>
       <family val="3"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -444,11 +438,10 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -456,20 +449,16 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -749,14 +738,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G23"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" customWidth="1"/>
-    <col min="2" max="2" width="62.85546875" style="1" customWidth="1"/>
-    <col min="3" max="8" width="20.42578125" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" customWidth="1"/>
+    <col min="2" max="2" width="62.88671875" style="1" customWidth="1"/>
+    <col min="3" max="8" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -779,88 +768,88 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>111</v>
+        <v>60</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>105</v>
       </c>
       <c r="C2" t="s">
         <v>9</v>
       </c>
       <c r="F2" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>112</v>
+        <v>61</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>106</v>
       </c>
       <c r="C3" t="s">
         <v>9</v>
       </c>
       <c r="F3" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G3" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="C4" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>110</v>
-      </c>
-      <c r="B5" s="9" t="s">
-        <v>113</v>
+        <v>104</v>
+      </c>
+      <c r="B5" t="s">
+        <v>107</v>
       </c>
       <c r="C5" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F6" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G6" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -869,18 +858,18 @@
         <v>15</v>
       </c>
       <c r="F7" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G7" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="C8" t="s">
         <v>10</v>
@@ -889,18 +878,18 @@
         <v>15</v>
       </c>
       <c r="F8" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G8" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
         <v>10</v>
@@ -909,110 +898,110 @@
         <v>16</v>
       </c>
       <c r="F9" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C10" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>14</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C11" t="s">
         <v>9</v>
       </c>
       <c r="F11" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="G11" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C12" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D12" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F12" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
       <c r="B13" t="s">
-        <v>85</v>
-      </c>
-      <c r="C13" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>10</v>
       </c>
       <c r="D13" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="F13" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="G13" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B14" t="s">
-        <v>74</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
         <v>9</v>
       </c>
       <c r="F15" t="s">
-        <v>108</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B23" s="8"/>
+        <v>102</v>
+      </c>
+      <c r="G15" s="3" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B23" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1023,105 +1012,105 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B5">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B6">
         <v>9</v>
       </c>
       <c r="C6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="B7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C7" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>80</v>
+      </c>
+      <c r="B8" t="s">
+        <v>84</v>
+      </c>
+      <c r="C8" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>80</v>
+      </c>
+      <c r="B9" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" t="s">
         <v>86</v>
-      </c>
-      <c r="B7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C7" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>86</v>
-      </c>
-      <c r="B8" t="s">
-        <v>90</v>
-      </c>
-      <c r="C8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>86</v>
-      </c>
-      <c r="B9" t="s">
-        <v>93</v>
-      </c>
-      <c r="C9" t="s">
-        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -1132,12 +1121,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="24.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -1169,7 +1158,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>36</v>
       </c>
@@ -1189,7 +1178,7 @@
         <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H2" t="s">
         <v>39</v>
@@ -1198,10 +1187,10 @@
         <v>42</v>
       </c>
       <c r="J2" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>36</v>
       </c>
@@ -1221,7 +1210,7 @@
         <v>41</v>
       </c>
       <c r="G3" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="H3" t="s">
         <v>39</v>
@@ -1230,27 +1219,30 @@
         <v>42</v>
       </c>
       <c r="J3" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>114</v>
+        <v>108</v>
       </c>
       <c r="B4" t="s">
-        <v>115</v>
+        <v>109</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="D4" t="s">
         <v>39</v>
       </c>
       <c r="E4" t="s">
-        <v>62</v>
+        <v>56</v>
+      </c>
+      <c r="F4" t="s">
+        <v>115</v>
       </c>
       <c r="G4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H4" t="s">
         <v>39</v>
@@ -1259,24 +1251,27 @@
         <v>42</v>
       </c>
       <c r="J4" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D5" t="s">
         <v>39</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>59</v>
+      </c>
+      <c r="F5" t="s">
+        <v>116</v>
       </c>
       <c r="G5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="H5" t="s">
         <v>39</v>
@@ -1285,50 +1280,47 @@
         <v>42</v>
       </c>
       <c r="J5" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>111</v>
+      </c>
+      <c r="C6" t="s">
+        <v>112</v>
       </c>
       <c r="D6" t="s">
         <v>39</v>
       </c>
       <c r="E6" t="s">
-        <v>46</v>
+        <v>113</v>
+      </c>
+      <c r="F6" t="s">
+        <v>114</v>
       </c>
       <c r="G6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
         <v>39</v>
       </c>
-      <c r="I6" t="s">
-        <v>42</v>
-      </c>
       <c r="J6" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="D7" t="s">
         <v>39</v>
       </c>
-      <c r="E7" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>58</v>
+      <c r="E7" t="s">
+        <v>45</v>
       </c>
       <c r="G7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="H7" t="s">
         <v>39</v>
@@ -1337,13 +1329,11 @@
         <v>42</v>
       </c>
       <c r="J7" t="s">
-        <v>43</v>
+        <v>110</v>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="E7" r:id="rId1" xr:uid="{CA295046-575D-408C-95E4-5B2B4E4C4C5B}"/>
-  </hyperlinks>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1351,12 +1341,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B12"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>17</v>
       </c>
@@ -1364,92 +1354,92 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="B2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B3" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="B4" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="B5" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="B7" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="7" t="s">
-        <v>102</v>
+    <row r="9" spans="1:2" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A9" s="5" t="s">
+        <v>96</v>
       </c>
       <c r="B9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="B10" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="B12" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
     </row>
   </sheetData>
@@ -1460,9 +1450,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E1"/>
-  <sheetFormatPr defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="10.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>21</v>
       </c>

</xml_diff>